<commit_message>
docs(arena): update benchmarks, dependencies and dates across all arenas
- Update intelligent-research-system ranking from #2 to #3 with new DeepResearch Bench score 53.54
- Replace GLM-5/Metaso MCP references with DeepSeek V4 Pro/StepSearch MCP
- Update "Last Updated" dates to 2026-05-18 and remove "Last Reviewed" field
- Simplify update_date.py to only update modification dates
- Add StepSearch MCP config step in tech-configuration docs
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -442,14 +442,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>私部署版：Claude Code + GLM 5 + Metaso</t>
+          <t>私部署版：Claude Code + DeepSeek V4 Pro + StepSearch</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Claude Code (by Anthropic) GitHub：https://github.com/anthropics/claude-code
-Metaso MCP (by 秘塔科技) 文档：https://www.modelscope.cn/mcp/servers/metasota/metaso-search
-GLM-5(by 智谱) GitHub：https://github.com/zai-org/GLM-5</t>
+StepSearch MCP (by 阶跃星辰) 文档：https://platform.stepfun.com/docs/zh/step-plan/integrations/search-mcp
+DeepSeek-V4-Pro(by 深度求索) Hugging Face：https://huggingface.co/deepseek-ai/DeepSeek-V4-Pro</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -494,7 +494,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>私部署版：Claude Code + DeepSeek V4 Pro/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6+ Metaso</t>
+          <t>私部署版：Hermes Agent + MiMo V2.5 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6+ Metaso</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">

</xml_diff>

<commit_message>
refactor(arena): move champion/challenger to common JSON and update model references
- Move champion and challenger fields from per-locale (en/zh) JSON into page.common.json
- Update challenger model references across arenas (e.g. Qwen 3.6 → Qwen 3.7)
- Update xlsx_to_json.py to extract champion/challenger into common fields
- Sync static-data.ts and export script with new data structure
- Regenerate arena-content.json and arenas.json from updated sources
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>私部署版：Hermes Agent + MiMo V2.5 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6+ Metaso</t>
+          <t>私部署版：Hermes Agent + Qwen 3.7/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6+ Metaso</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -579,7 +579,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>云端版：Lovable + DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6/Minimax M2.7 + Claude Code</t>
+          <t>云端版：Lovable + Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7 + Claude Code</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>私部署版：LangChain + DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain + Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N4"/>
@@ -745,7 +745,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>私部署版：OpenClaw + DeepSeek V4 Pro/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6  + FFmpeg + Qwen3-ASR + Qwen3-TTS</t>
+          <t>私部署版：OpenClaw + Qwen 3.7/DeepSeek V4 Pro/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6  + FFmpeg + FireRedASR/Qwen3-ASR/GLM-ASR + Qwen3-TTS/Fun-CosyVoice 3.0/GLM-TTS</t>
         </is>
       </c>
       <c r="N5"/>
@@ -817,7 +817,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>私部署版：BISHENG + DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6/Minimax M2.7</t>
+          <t>私部署版：BISHENG + Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7</t>
         </is>
       </c>
       <c r="N6"/>
@@ -962,7 +962,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>私部署版：Claude Code + DeepSeek V4 Pro/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6</t>
+          <t>私部署版：Claude Code + Qwen 3.7/DeepSeek V4 Pro/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6</t>
         </is>
       </c>
       <c r="N8"/>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>私部署版：Coze +  DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6</t>
+          <t>私部署版：Coze +  Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6</t>
         </is>
       </c>
       <c r="N12"/>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>私部署版：LangChain +  DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain +  Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N13"/>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>私部署版：LangChain +  DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain +  Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N14"/>

</xml_diff>

<commit_message>
docs(arena): update dates to 2026-06-01 across all arenas
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -579,7 +579,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>云端版：Lovable + Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7 + Claude Code</t>
+          <t>云端版：Lovable + MiniMax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6 + Claude Code</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>私部署版：LangChain + Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain + Minimax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N4"/>
@@ -817,7 +817,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>私部署版：BISHENG + Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7</t>
+          <t>私部署版：BISHENG + Minimax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Hy3 preview/Step 3.7 Flash</t>
         </is>
       </c>
       <c r="N6"/>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>私部署版：Coze +  Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6</t>
+          <t>私部署版：Coze +  Minimax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6</t>
         </is>
       </c>
       <c r="N12"/>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>私部署版：LangChain +  Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain +  Minimax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N13"/>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>私部署版：LangChain +  Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain +  Minimax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N14"/>

</xml_diff>

<commit_message>
docs(arena): update dates to 2026-06-08 across all arenas
- Sync 最近更新/Last Updated from 2026-06-01 to 2026-06-08 in all 13 arena overviews and main docs
- Update List of Arenas.csv and page.common.json with the new date
- Binary update for List of Arenas.xlsx
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -817,7 +817,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>私部署版：BISHENG + Minimax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Hy3 preview/Step 3.7 Flash</t>
+          <t>私部署版：BISHENG + Minimax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Hy3 preview/Step 3.7 Flash/Ling 2.6 flash</t>
         </is>
       </c>
       <c r="N6"/>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>寻找攻擂者</t>
+          <t>私部署版：Ultralytics YOLO （YOLO 26）+ Triton + Perf Analyzer</t>
         </is>
       </c>
       <c r="N10"/>

</xml_diff>

<commit_message>
update arena: sync dates to 2026-06-15 and content updates
- update overview/main.md dates across 13 arenas (2026-06-08 -> 2026-06-15)
- update List of Arenas.csv schema and page.common.json
- add sync-arena script and stage it in .gitignore
- update package.json with new sync script entry
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>私部署版：Hermes Agent + Qwen 3.7/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6+ Metaso</t>
+          <t>私部署版：Hermes Agent + GLM 5.2/Qwen 3.7/MiMo V2.5 Pro/Kimi K2.6+ Metaso</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -579,7 +579,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>云端版：Lovable + MiniMax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6 + Claude Code</t>
+          <t>云端版：Lovable + Kimi K2.7 Code/GLM 5.2/MiniMax M3/Qwen 3.7/DeepSeek V4 Pro/Kimi K2.6 + Claude Code</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>私部署版：LangChain + Minimax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain + GLM 5.2/Minimax M3/Qwen 3.7/DeepSeek V4 Pro/Kimi K2.6  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N4"/>
@@ -745,7 +745,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>私部署版：OpenClaw + Qwen 3.7/DeepSeek V4 Pro/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6  + FFmpeg + FireRedASR/Qwen3-ASR/GLM-ASR + Qwen3-TTS/Fun-CosyVoice 3.0/GLM-TTS</t>
+          <t>私部署版：OpenClaw + Kimi K2.7 Code/GLM 5.2/Qwen 3.7/DeepSeek V4 Pro/MiMo V2.5 Pro/Kimi K2.6  + FFmpeg + FireRedASR/Qwen3-ASR/GLM-ASR + VoxCPM/Qwen3-TTS/Fun-CosyVoice 3.0/GLM-TTS</t>
         </is>
       </c>
       <c r="N5"/>
@@ -817,7 +817,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>私部署版：BISHENG + Minimax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Hy3 preview/Step 3.7 Flash/Ling 2.6 flash</t>
+          <t>私部署版：BISHENG + GLM 5.2/Minimax M3/Qwen 3.7/DeepSeek V4 Pro/Kimi K2.6/Hy3 preview/Step 3.7 Flash/Ling 2.6 flash</t>
         </is>
       </c>
       <c r="N6"/>
@@ -962,7 +962,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>私部署版：Claude Code + Qwen 3.7/DeepSeek V4 Pro/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6</t>
+          <t>私部署版：Claude Code + GLM 5.2/Kimi K2.7 Code/Qwen 3.7/DeepSeek V4 Pro/MiMo V2.5 Pro/Kimi K2.6</t>
         </is>
       </c>
       <c r="N8"/>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>私部署版：Coze +  Minimax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6</t>
+          <t>私部署版：Coze +  GLM 5.2/Minimax M3/Qwen 3.7/DeepSeek V4 Pro/Kimi K2.6</t>
         </is>
       </c>
       <c r="N12"/>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>私部署版：LangChain +  Minimax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain +  GLM 5.2/Minimax M3/Qwen 3.7/DeepSeek V4 Pro/Kimi K2.6  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N13"/>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>私部署版：LangChain +  Minimax M3/Qwen 3.7/DeepSeek V4 Pro/GLM 5.1/Kimi K2.6  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain +  Kimi K2.7 Code/GLM 5.2/Minimax M3/Qwen 3.7/DeepSeek V4 Pro/Kimi K2.6  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N14"/>

</xml_diff>